<commit_message>
Atualiza dados do Google Trends
</commit_message>
<xml_diff>
--- a/data/dados.xlsx
+++ b/data/dados.xlsx
@@ -3936,7 +3936,7 @@
         <v>29</v>
       </c>
       <c r="G67">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="H67" t="s">
         <v>36</v>
@@ -4794,7 +4794,7 @@
         <v>30</v>
       </c>
       <c r="G100">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H100" t="s">
         <v>36</v>
@@ -5652,7 +5652,7 @@
         <v>31</v>
       </c>
       <c r="G133">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H133" t="s">
         <v>36</v>
@@ -6588,7 +6588,7 @@
         <v>33</v>
       </c>
       <c r="G169">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H169" t="s">
         <v>36</v>
@@ -6640,7 +6640,7 @@
         <v>33</v>
       </c>
       <c r="G171">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H171" t="s">
         <v>36</v>
@@ -6848,7 +6848,7 @@
         <v>33</v>
       </c>
       <c r="G179">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H179" t="s">
         <v>36</v>
@@ -6926,7 +6926,7 @@
         <v>33</v>
       </c>
       <c r="G182">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H182" t="s">
         <v>36</v>
@@ -7108,7 +7108,7 @@
         <v>33</v>
       </c>
       <c r="G189">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H189" t="s">
         <v>36</v>
@@ -7212,7 +7212,7 @@
         <v>33</v>
       </c>
       <c r="G193">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H193" t="s">
         <v>36</v>
@@ -7368,7 +7368,7 @@
         <v>33</v>
       </c>
       <c r="G199">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="H199" t="s">
         <v>36</v>
@@ -8226,7 +8226,7 @@
         <v>34</v>
       </c>
       <c r="G232">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H232" t="s">
         <v>36</v>
@@ -9175,22 +9175,22 @@
         <v>50.77777777777778</v>
       </c>
       <c r="D3">
-        <v>47.11111111111111</v>
+        <v>46.88888888888889</v>
       </c>
       <c r="E3">
-        <v>-0.07221006564551413</v>
+        <v>-0.07658643326039394</v>
       </c>
       <c r="F3">
-        <v>36</v>
+        <v>35.33333333333334</v>
       </c>
       <c r="G3">
         <v>29.66666666666667</v>
       </c>
       <c r="H3">
-        <v>0.2134831460674156</v>
+        <v>0.1910112359550562</v>
       </c>
       <c r="I3">
-        <v>0.4230970861543641</v>
+        <v>0.4238783724201226</v>
       </c>
       <c r="J3" t="s">
         <v>46</v>
@@ -9207,22 +9207,22 @@
         <v>55.88888888888889</v>
       </c>
       <c r="D4">
-        <v>38</v>
+        <v>38.11111111111111</v>
       </c>
       <c r="E4">
-        <v>-0.320079522862823</v>
+        <v>-0.3180914512922465</v>
       </c>
       <c r="F4">
-        <v>25.33333333333333</v>
+        <v>25.66666666666667</v>
       </c>
       <c r="G4">
         <v>31.66666666666667</v>
       </c>
       <c r="H4">
-        <v>-0.2000000000000001</v>
+        <v>-0.1894736842105263</v>
       </c>
       <c r="I4">
-        <v>0.38968929931421</v>
+        <v>0.3888486146797661</v>
       </c>
       <c r="J4" t="s">
         <v>47</v>
@@ -9239,22 +9239,22 @@
         <v>50.44444444444444</v>
       </c>
       <c r="D5">
-        <v>69.22222222222223</v>
+        <v>69</v>
       </c>
       <c r="E5">
-        <v>0.3722466960352424</v>
+        <v>0.36784140969163</v>
       </c>
       <c r="F5">
-        <v>65</v>
+        <v>64.33333333333333</v>
       </c>
       <c r="G5">
         <v>61</v>
       </c>
       <c r="H5">
-        <v>0.06557377049180335</v>
+        <v>0.05464480874316924</v>
       </c>
       <c r="I5">
-        <v>0.7894911189938829</v>
+        <v>0.7890870428085769</v>
       </c>
       <c r="J5" t="s">
         <v>46</v>
@@ -9303,22 +9303,22 @@
         <v>55</v>
       </c>
       <c r="D7">
-        <v>72.11111111111111</v>
+        <v>72.55555555555556</v>
       </c>
       <c r="E7">
-        <v>0.3111111111111111</v>
+        <v>0.3191919191919192</v>
       </c>
       <c r="F7">
-        <v>51.33333333333334</v>
+        <v>53</v>
       </c>
       <c r="G7">
         <v>73.66666666666667</v>
       </c>
       <c r="H7">
-        <v>-0.3031674208144797</v>
+        <v>-0.2805429864253394</v>
       </c>
       <c r="I7">
-        <v>0.273667644759039</v>
+        <v>0.2705889226732273</v>
       </c>
       <c r="J7" t="s">
         <v>47</v>
@@ -9335,22 +9335,22 @@
         <v>26.77777777777778</v>
       </c>
       <c r="D8">
-        <v>38.33333333333334</v>
+        <v>38.44444444444444</v>
       </c>
       <c r="E8">
-        <v>0.4315352697095436</v>
+        <v>0.4356846473029046</v>
       </c>
       <c r="F8">
-        <v>29.66666666666667</v>
+        <v>30</v>
       </c>
       <c r="G8">
         <v>23.66666666666667</v>
       </c>
       <c r="H8">
-        <v>0.2535211267605633</v>
+        <v>0.2676056338028168</v>
       </c>
       <c r="I8">
-        <v>0.6275203823400812</v>
+        <v>0.6273275480689409</v>
       </c>
       <c r="J8" t="s">
         <v>46</v>
@@ -9494,40 +9494,40 @@
         <v>29</v>
       </c>
       <c r="C3">
-        <v>1.723160027008778</v>
+        <v>1.725490196078431</v>
       </c>
       <c r="D3">
-        <v>1.255232950708981</v>
+        <v>1.256930358350237</v>
       </c>
       <c r="E3">
-        <v>1.032410533423363</v>
+        <v>1.033806626098715</v>
       </c>
       <c r="F3">
-        <v>0.7947332883187036</v>
+        <v>0.7958079783637592</v>
       </c>
       <c r="G3">
-        <v>0.6907494935854153</v>
+        <v>0.691683569979716</v>
       </c>
       <c r="H3">
-        <v>0.6090479405806888</v>
+        <v>0.6098715348208248</v>
       </c>
       <c r="I3">
-        <v>0.824442943956786</v>
+        <v>0.8255578093306287</v>
       </c>
       <c r="J3">
-        <v>0.7873058744091831</v>
+        <v>0.7883705206220419</v>
       </c>
       <c r="K3">
-        <v>0.8541525995948684</v>
+        <v>0.8404327248140635</v>
       </c>
       <c r="L3">
-        <v>0.9469952734638758</v>
+        <v>0.9482758620689655</v>
       </c>
       <c r="M3">
-        <v>1.147535449020932</v>
+        <v>1.149087221095335</v>
       </c>
       <c r="N3">
-        <v>1.548615800135044</v>
+        <v>1.550709939148073</v>
       </c>
     </row>
     <row r="4" spans="1:14">
@@ -9538,40 +9538,40 @@
         <v>30</v>
       </c>
       <c r="C4">
-        <v>1.635333333333333</v>
+        <v>1.634243837441705</v>
       </c>
       <c r="D4">
-        <v>1.584</v>
+        <v>1.582944703530979</v>
       </c>
       <c r="E4">
-        <v>0.9533333333333334</v>
+        <v>0.9526982011992006</v>
       </c>
       <c r="F4">
-        <v>0.7406666666666666</v>
+        <v>0.7401732178547634</v>
       </c>
       <c r="G4">
-        <v>0.8066666666666666</v>
+        <v>0.8061292471685543</v>
       </c>
       <c r="H4">
-        <v>0.7040000000000001</v>
+        <v>0.703530979347102</v>
       </c>
       <c r="I4">
-        <v>0.8360000000000001</v>
+        <v>0.8354430379746836</v>
       </c>
       <c r="J4">
-        <v>0.6820000000000001</v>
+        <v>0.681545636242505</v>
       </c>
       <c r="K4">
-        <v>0.858</v>
+        <v>0.8647568287808128</v>
       </c>
       <c r="L4">
-        <v>1.056</v>
+        <v>1.055296469020653</v>
       </c>
       <c r="M4">
-        <v>1.078</v>
+        <v>1.07728181212525</v>
       </c>
       <c r="N4">
-        <v>1.166</v>
+        <v>1.165223184543638</v>
       </c>
     </row>
     <row r="5" spans="1:14">
@@ -9582,40 +9582,40 @@
         <v>31</v>
       </c>
       <c r="C5">
-        <v>0.8258258258258259</v>
+        <v>0.8270676691729324</v>
       </c>
       <c r="D5">
-        <v>1.106606606606606</v>
+        <v>1.108270676691729</v>
       </c>
       <c r="E5">
-        <v>1.106606606606606</v>
+        <v>1.108270676691729</v>
       </c>
       <c r="F5">
-        <v>0.9084084084084083</v>
+        <v>0.9097744360902255</v>
       </c>
       <c r="G5">
-        <v>1.304804804804805</v>
+        <v>1.306766917293233</v>
       </c>
       <c r="H5">
-        <v>0.8588588588588587</v>
+        <v>0.8601503759398496</v>
       </c>
       <c r="I5">
-        <v>1.156156156156156</v>
+        <v>1.157894736842105</v>
       </c>
       <c r="J5">
-        <v>0.801051051051051</v>
+        <v>0.8022556390977444</v>
       </c>
       <c r="K5">
-        <v>1.197447447447447</v>
+        <v>1.182706766917293</v>
       </c>
       <c r="L5">
-        <v>0.5326576576576576</v>
+        <v>0.5334586466165413</v>
       </c>
       <c r="M5">
-        <v>0.9786036036036035</v>
+        <v>0.9800751879699248</v>
       </c>
       <c r="N5">
-        <v>1.09009009009009</v>
+        <v>1.091729323308271</v>
       </c>
     </row>
     <row r="6" spans="1:14">
@@ -9670,40 +9670,40 @@
         <v>33</v>
       </c>
       <c r="C7">
-        <v>1.056692913385827</v>
+        <v>1.061909758656873</v>
       </c>
       <c r="D7">
-        <v>1.224146981627297</v>
+        <v>1.223504721930745</v>
       </c>
       <c r="E7">
-        <v>1.195275590551181</v>
+        <v>1.183105981112277</v>
       </c>
       <c r="F7">
-        <v>0.9758530183727034</v>
+        <v>0.9695697796432319</v>
       </c>
       <c r="G7">
-        <v>1.039370078740157</v>
+        <v>1.03305351521511</v>
       </c>
       <c r="H7">
-        <v>0.9412073490813648</v>
+        <v>0.9407135362014691</v>
       </c>
       <c r="I7">
-        <v>1.056692913385827</v>
+        <v>1.056138509968521</v>
       </c>
       <c r="J7">
-        <v>0.8661417322834646</v>
+        <v>0.8656873032528857</v>
       </c>
       <c r="K7">
-        <v>0.7564304461942257</v>
+        <v>0.7848898216159497</v>
       </c>
       <c r="L7">
-        <v>0.6755905511811023</v>
+        <v>0.6752360965372508</v>
       </c>
       <c r="M7">
-        <v>1.013385826771654</v>
+        <v>1.004197271773347</v>
       </c>
       <c r="N7">
-        <v>1.143307086614173</v>
+        <v>1.142707240293809</v>
       </c>
     </row>
     <row r="8" spans="1:14">
@@ -9714,40 +9714,40 @@
         <v>34</v>
       </c>
       <c r="C8">
-        <v>1.165942658557776</v>
+        <v>1.164930555555556</v>
       </c>
       <c r="D8">
-        <v>2.054735013032146</v>
+        <v>2.052951388888889</v>
       </c>
       <c r="E8">
-        <v>0.9079061685490879</v>
+        <v>0.9071180555555557</v>
       </c>
       <c r="F8">
-        <v>0.9748045178105996</v>
+        <v>0.9739583333333334</v>
       </c>
       <c r="G8">
-        <v>0.9079061685490879</v>
+        <v>0.9071180555555557</v>
       </c>
       <c r="H8">
-        <v>0.420503909643788</v>
+        <v>0.4201388888888889</v>
       </c>
       <c r="I8">
-        <v>0.8887923544743702</v>
+        <v>0.8880208333333334</v>
       </c>
       <c r="J8">
-        <v>1.156385751520417</v>
+        <v>1.155381944444445</v>
       </c>
       <c r="K8">
-        <v>1.137271937445699</v>
+        <v>1.145833333333333</v>
       </c>
       <c r="L8">
-        <v>0.6020851433536056</v>
+        <v>0.6015625</v>
       </c>
       <c r="M8">
-        <v>0.4874022589052998</v>
+        <v>0.4869791666666667</v>
       </c>
       <c r="N8">
-        <v>0.9891398783666379</v>
+        <v>0.9882812500000001</v>
       </c>
     </row>
     <row r="9" spans="1:14">
@@ -10439,7 +10439,7 @@
         <v>46082</v>
       </c>
       <c r="E28">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F28">
         <v>2026</v>
@@ -15847,22 +15847,22 @@
         <v>29</v>
       </c>
       <c r="C3">
-        <v>47.11111111111111</v>
+        <v>46.88888888888889</v>
       </c>
       <c r="D3">
-        <v>-0.07221006564551413</v>
+        <v>-0.07658643326039394</v>
       </c>
       <c r="E3">
-        <v>0.2134831460674156</v>
+        <v>0.1910112359550562</v>
       </c>
       <c r="F3">
-        <v>0.4230970861543641</v>
+        <v>0.4238783724201226</v>
       </c>
       <c r="G3">
         <v>1</v>
       </c>
       <c r="H3">
-        <v>1.723160027008778</v>
+        <v>1.725490196078431</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -15873,22 +15873,22 @@
         <v>30</v>
       </c>
       <c r="C4">
-        <v>38</v>
+        <v>38.11111111111111</v>
       </c>
       <c r="D4">
-        <v>-0.320079522862823</v>
+        <v>-0.3180914512922465</v>
       </c>
       <c r="E4">
-        <v>-0.2000000000000001</v>
+        <v>-0.1894736842105263</v>
       </c>
       <c r="F4">
-        <v>0.38968929931421</v>
+        <v>0.3888486146797661</v>
       </c>
       <c r="G4">
         <v>1</v>
       </c>
       <c r="H4">
-        <v>1.635333333333333</v>
+        <v>1.634243837441705</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -15899,22 +15899,22 @@
         <v>31</v>
       </c>
       <c r="C5">
-        <v>69.22222222222223</v>
+        <v>69</v>
       </c>
       <c r="D5">
-        <v>0.3722466960352424</v>
+        <v>0.36784140969163</v>
       </c>
       <c r="E5">
-        <v>0.06557377049180335</v>
+        <v>0.05464480874316924</v>
       </c>
       <c r="F5">
-        <v>0.7894911189938829</v>
+        <v>0.7890870428085769</v>
       </c>
       <c r="G5">
         <v>5</v>
       </c>
       <c r="H5">
-        <v>1.304804804804805</v>
+        <v>1.306766917293233</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -15951,22 +15951,22 @@
         <v>33</v>
       </c>
       <c r="C7">
-        <v>72.11111111111111</v>
+        <v>72.55555555555556</v>
       </c>
       <c r="D7">
-        <v>0.3111111111111111</v>
+        <v>0.3191919191919192</v>
       </c>
       <c r="E7">
-        <v>-0.3031674208144797</v>
+        <v>-0.2805429864253394</v>
       </c>
       <c r="F7">
-        <v>0.273667644759039</v>
+        <v>0.2705889226732273</v>
       </c>
       <c r="G7">
         <v>2</v>
       </c>
       <c r="H7">
-        <v>1.224146981627297</v>
+        <v>1.223504721930745</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -15977,22 +15977,22 @@
         <v>34</v>
       </c>
       <c r="C8">
-        <v>38.33333333333334</v>
+        <v>38.44444444444444</v>
       </c>
       <c r="D8">
-        <v>0.4315352697095436</v>
+        <v>0.4356846473029046</v>
       </c>
       <c r="E8">
-        <v>0.2535211267605633</v>
+        <v>0.2676056338028168</v>
       </c>
       <c r="F8">
-        <v>0.6275203823400812</v>
+        <v>0.6273275480689409</v>
       </c>
       <c r="G8">
         <v>2</v>
       </c>
       <c r="H8">
-        <v>2.054735013032146</v>
+        <v>2.052951388888889</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -29811,7 +29811,7 @@
         <v>28</v>
       </c>
       <c r="F2">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G2">
         <v>9</v>
@@ -29834,10 +29834,10 @@
         <v>28</v>
       </c>
       <c r="F3">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G3">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -29857,7 +29857,7 @@
         <v>28</v>
       </c>
       <c r="F4">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G4">
         <v>7</v>
@@ -29880,7 +29880,7 @@
         <v>28</v>
       </c>
       <c r="F5">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G5">
         <v>7</v>
@@ -29903,7 +29903,7 @@
         <v>28</v>
       </c>
       <c r="F6">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G6">
         <v>7</v>
@@ -29926,7 +29926,7 @@
         <v>28</v>
       </c>
       <c r="F7">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G7">
         <v>7</v>
@@ -29949,10 +29949,10 @@
         <v>28</v>
       </c>
       <c r="F8">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="G8">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -29972,7 +29972,7 @@
         <v>28</v>
       </c>
       <c r="F9">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="G9">
         <v>9</v>
@@ -29995,7 +29995,7 @@
         <v>28</v>
       </c>
       <c r="F10">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G10">
         <v>9</v>
@@ -30018,10 +30018,10 @@
         <v>28</v>
       </c>
       <c r="F11">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G11">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -30041,7 +30041,7 @@
         <v>28</v>
       </c>
       <c r="F12">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G12">
         <v>8</v>
@@ -30067,7 +30067,7 @@
         <v>21</v>
       </c>
       <c r="G13">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -30087,7 +30087,7 @@
         <v>28</v>
       </c>
       <c r="F14">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G14">
         <v>9</v>
@@ -30110,7 +30110,7 @@
         <v>28</v>
       </c>
       <c r="F15">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G15">
         <v>10</v>
@@ -30156,7 +30156,7 @@
         <v>28</v>
       </c>
       <c r="F17">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G17">
         <v>9</v>
@@ -30179,7 +30179,7 @@
         <v>28</v>
       </c>
       <c r="F18">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="G18">
         <v>8</v>
@@ -30202,7 +30202,7 @@
         <v>28</v>
       </c>
       <c r="F19">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G19">
         <v>8</v>
@@ -30225,7 +30225,7 @@
         <v>28</v>
       </c>
       <c r="F20">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G20">
         <v>10</v>
@@ -30248,7 +30248,7 @@
         <v>28</v>
       </c>
       <c r="F21">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G21">
         <v>10</v>
@@ -30271,7 +30271,7 @@
         <v>28</v>
       </c>
       <c r="F22">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G22">
         <v>9</v>
@@ -30294,7 +30294,7 @@
         <v>28</v>
       </c>
       <c r="F23">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G23">
         <v>8</v>
@@ -30317,10 +30317,10 @@
         <v>28</v>
       </c>
       <c r="F24">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G24">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -30340,7 +30340,7 @@
         <v>28</v>
       </c>
       <c r="F25">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G25">
         <v>11</v>
@@ -30363,10 +30363,10 @@
         <v>28</v>
       </c>
       <c r="F26">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G26">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -30409,7 +30409,7 @@
         <v>28</v>
       </c>
       <c r="F28">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G28">
         <v>10</v>
@@ -30432,7 +30432,7 @@
         <v>28</v>
       </c>
       <c r="F29">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G29">
         <v>10</v>
@@ -30455,10 +30455,10 @@
         <v>28</v>
       </c>
       <c r="F30">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G30">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -30478,10 +30478,10 @@
         <v>28</v>
       </c>
       <c r="F31">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G31">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="32" spans="1:7">
@@ -30501,7 +30501,7 @@
         <v>28</v>
       </c>
       <c r="F32">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G32">
         <v>10</v>
@@ -30524,10 +30524,10 @@
         <v>28</v>
       </c>
       <c r="F33">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G33">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -30547,7 +30547,7 @@
         <v>28</v>
       </c>
       <c r="F34">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G34">
         <v>7</v>
@@ -30570,10 +30570,10 @@
         <v>29</v>
       </c>
       <c r="F35">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="G35">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -30593,10 +30593,10 @@
         <v>29</v>
       </c>
       <c r="F36">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="G36">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -30616,10 +30616,10 @@
         <v>29</v>
       </c>
       <c r="F37">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G37">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="38" spans="1:7">
@@ -30639,10 +30639,10 @@
         <v>29</v>
       </c>
       <c r="F38">
-        <v>83</v>
+        <v>59</v>
       </c>
       <c r="G38">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -30662,10 +30662,10 @@
         <v>29</v>
       </c>
       <c r="F39">
-        <v>90</v>
+        <v>36</v>
       </c>
       <c r="G39">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -30685,10 +30685,10 @@
         <v>29</v>
       </c>
       <c r="F40">
-        <v>95</v>
+        <v>39</v>
       </c>
       <c r="G40">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="41" spans="1:7">
@@ -30708,10 +30708,10 @@
         <v>29</v>
       </c>
       <c r="F41">
-        <v>59</v>
+        <v>33</v>
       </c>
       <c r="G41">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="42" spans="1:7">
@@ -30731,10 +30731,10 @@
         <v>29</v>
       </c>
       <c r="F42">
-        <v>73</v>
+        <v>36</v>
       </c>
       <c r="G42">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="43" spans="1:7">
@@ -30754,10 +30754,10 @@
         <v>29</v>
       </c>
       <c r="F43">
-        <v>78</v>
+        <v>45</v>
       </c>
       <c r="G43">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="44" spans="1:7">
@@ -30777,10 +30777,10 @@
         <v>29</v>
       </c>
       <c r="F44">
-        <v>69</v>
+        <v>46</v>
       </c>
       <c r="G44">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="45" spans="1:7">
@@ -30800,10 +30800,10 @@
         <v>29</v>
       </c>
       <c r="F45">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="G45">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="46" spans="1:7">
@@ -30823,10 +30823,10 @@
         <v>29</v>
       </c>
       <c r="F46">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="G46">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
     <row r="47" spans="1:7">
@@ -30846,10 +30846,10 @@
         <v>29</v>
       </c>
       <c r="F47">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="G47">
-        <v>20</v>
+        <v>35</v>
       </c>
     </row>
     <row r="48" spans="1:7">
@@ -30869,10 +30869,10 @@
         <v>29</v>
       </c>
       <c r="F48">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G48">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
     <row r="49" spans="1:7">
@@ -30892,10 +30892,10 @@
         <v>29</v>
       </c>
       <c r="F49">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="G49">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="50" spans="1:7">
@@ -30915,10 +30915,10 @@
         <v>29</v>
       </c>
       <c r="F50">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="G50">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="51" spans="1:7">
@@ -30938,10 +30938,10 @@
         <v>29</v>
       </c>
       <c r="F51">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="G51">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="52" spans="1:7">
@@ -30961,10 +30961,10 @@
         <v>29</v>
       </c>
       <c r="F52">
-        <v>68</v>
+        <v>40</v>
       </c>
       <c r="G52">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="53" spans="1:7">
@@ -30984,10 +30984,10 @@
         <v>29</v>
       </c>
       <c r="F53">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="G53">
-        <v>11</v>
+        <v>19</v>
       </c>
     </row>
     <row r="54" spans="1:7">
@@ -31007,10 +31007,10 @@
         <v>29</v>
       </c>
       <c r="F54">
-        <v>64</v>
+        <v>43</v>
       </c>
       <c r="G54">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="55" spans="1:7">
@@ -31030,10 +31030,10 @@
         <v>29</v>
       </c>
       <c r="F55">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="G55">
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
     <row r="56" spans="1:7">
@@ -31053,10 +31053,10 @@
         <v>29</v>
       </c>
       <c r="F56">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="G56">
-        <v>13</v>
+        <v>22</v>
       </c>
     </row>
     <row r="57" spans="1:7">
@@ -31076,10 +31076,10 @@
         <v>29</v>
       </c>
       <c r="F57">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="G57">
-        <v>13</v>
+        <v>22</v>
       </c>
     </row>
     <row r="58" spans="1:7">
@@ -31099,10 +31099,10 @@
         <v>29</v>
       </c>
       <c r="F58">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="G58">
-        <v>19</v>
+        <v>31</v>
       </c>
     </row>
     <row r="59" spans="1:7">
@@ -31122,10 +31122,10 @@
         <v>29</v>
       </c>
       <c r="F59">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="G59">
-        <v>23</v>
+        <v>40</v>
       </c>
     </row>
     <row r="60" spans="1:7">
@@ -31145,10 +31145,10 @@
         <v>29</v>
       </c>
       <c r="F60">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="G60">
-        <v>17</v>
+        <v>28</v>
       </c>
     </row>
     <row r="61" spans="1:7">
@@ -31168,10 +31168,10 @@
         <v>29</v>
       </c>
       <c r="F61">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G61">
-        <v>13</v>
+        <v>22</v>
       </c>
     </row>
     <row r="62" spans="1:7">
@@ -31191,10 +31191,10 @@
         <v>29</v>
       </c>
       <c r="F62">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G62">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="63" spans="1:7">
@@ -31214,10 +31214,10 @@
         <v>29</v>
       </c>
       <c r="F63">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="G63">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="64" spans="1:7">
@@ -31237,10 +31237,10 @@
         <v>29</v>
       </c>
       <c r="F64">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="G64">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="65" spans="1:7">
@@ -31260,10 +31260,10 @@
         <v>29</v>
       </c>
       <c r="F65">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="G65">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="66" spans="1:7">
@@ -31283,10 +31283,10 @@
         <v>29</v>
       </c>
       <c r="F66">
-        <v>67</v>
+        <v>40</v>
       </c>
       <c r="G66">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="67" spans="1:7">
@@ -31306,10 +31306,10 @@
         <v>29</v>
       </c>
       <c r="F67">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="G67">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="68" spans="1:7">
@@ -31329,10 +31329,10 @@
         <v>30</v>
       </c>
       <c r="F68">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="G68">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="69" spans="1:7">
@@ -31375,10 +31375,10 @@
         <v>30</v>
       </c>
       <c r="F70">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G70">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="71" spans="1:7">
@@ -31398,10 +31398,10 @@
         <v>30</v>
       </c>
       <c r="F71">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="G71">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="72" spans="1:7">
@@ -31421,10 +31421,10 @@
         <v>30</v>
       </c>
       <c r="F72">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="G72">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="73" spans="1:7">
@@ -31444,7 +31444,7 @@
         <v>30</v>
       </c>
       <c r="F73">
-        <v>69</v>
+        <v>42</v>
       </c>
       <c r="G73">
         <v>14</v>
@@ -31467,7 +31467,7 @@
         <v>30</v>
       </c>
       <c r="F74">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="G74">
         <v>17</v>
@@ -31490,7 +31490,7 @@
         <v>30</v>
       </c>
       <c r="F75">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="G75">
         <v>17</v>
@@ -31513,10 +31513,10 @@
         <v>30</v>
       </c>
       <c r="F76">
-        <v>71</v>
+        <v>51</v>
       </c>
       <c r="G76">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="77" spans="1:7">
@@ -31536,10 +31536,10 @@
         <v>30</v>
       </c>
       <c r="F77">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="G77">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="78" spans="1:7">
@@ -31559,7 +31559,7 @@
         <v>30</v>
       </c>
       <c r="F78">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G78">
         <v>21</v>
@@ -31582,10 +31582,10 @@
         <v>30</v>
       </c>
       <c r="F79">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="G79">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="80" spans="1:7">
@@ -31605,10 +31605,10 @@
         <v>30</v>
       </c>
       <c r="F80">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="G80">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="81" spans="1:7">
@@ -31628,10 +31628,10 @@
         <v>30</v>
       </c>
       <c r="F81">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="G81">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="82" spans="1:7">
@@ -31651,10 +31651,10 @@
         <v>30</v>
       </c>
       <c r="F82">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="G82">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="83" spans="1:7">
@@ -31674,7 +31674,7 @@
         <v>30</v>
       </c>
       <c r="F83">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="G83">
         <v>20</v>
@@ -31697,10 +31697,10 @@
         <v>30</v>
       </c>
       <c r="F84">
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="G84">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="85" spans="1:7">
@@ -31720,7 +31720,7 @@
         <v>30</v>
       </c>
       <c r="F85">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="G85">
         <v>18</v>
@@ -31743,10 +31743,10 @@
         <v>30</v>
       </c>
       <c r="F86">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="G86">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="87" spans="1:7">
@@ -31766,10 +31766,10 @@
         <v>30</v>
       </c>
       <c r="F87">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="G87">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="88" spans="1:7">
@@ -31789,10 +31789,10 @@
         <v>30</v>
       </c>
       <c r="F88">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="G88">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="89" spans="1:7">
@@ -31812,7 +31812,7 @@
         <v>30</v>
       </c>
       <c r="F89">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="G89">
         <v>25</v>
@@ -31835,10 +31835,10 @@
         <v>30</v>
       </c>
       <c r="F90">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G90">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="91" spans="1:7">
@@ -31858,10 +31858,10 @@
         <v>30</v>
       </c>
       <c r="F91">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="G91">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="92" spans="1:7">
@@ -31881,10 +31881,10 @@
         <v>30</v>
       </c>
       <c r="F92">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="G92">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="93" spans="1:7">
@@ -31904,7 +31904,7 @@
         <v>30</v>
       </c>
       <c r="F93">
-        <v>81</v>
+        <v>61</v>
       </c>
       <c r="G93">
         <v>26</v>
@@ -31927,10 +31927,10 @@
         <v>30</v>
       </c>
       <c r="F94">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="G94">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="95" spans="1:7">
@@ -31950,10 +31950,10 @@
         <v>30</v>
       </c>
       <c r="F95">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G95">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="96" spans="1:7">
@@ -31973,7 +31973,7 @@
         <v>30</v>
       </c>
       <c r="F96">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G96">
         <v>16</v>
@@ -31996,10 +31996,10 @@
         <v>30</v>
       </c>
       <c r="F97">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="G97">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="98" spans="1:7">
@@ -32019,10 +32019,10 @@
         <v>30</v>
       </c>
       <c r="F98">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="G98">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="99" spans="1:7">
@@ -32042,7 +32042,7 @@
         <v>30</v>
       </c>
       <c r="F99">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="G99">
         <v>9</v>
@@ -32065,10 +32065,10 @@
         <v>30</v>
       </c>
       <c r="F100">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="G100">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="101" spans="1:7">
@@ -32088,7 +32088,7 @@
         <v>31</v>
       </c>
       <c r="F101">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="G101">
         <v>0</v>
@@ -32111,7 +32111,7 @@
         <v>31</v>
       </c>
       <c r="F102">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="G102">
         <v>0</v>
@@ -32134,10 +32134,10 @@
         <v>31</v>
       </c>
       <c r="F103">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="G103">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104" spans="1:7">
@@ -32157,7 +32157,7 @@
         <v>31</v>
       </c>
       <c r="F104">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="G104">
         <v>0</v>
@@ -32180,7 +32180,7 @@
         <v>31</v>
       </c>
       <c r="F105">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="G105">
         <v>0</v>
@@ -32203,7 +32203,7 @@
         <v>31</v>
       </c>
       <c r="F106">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="G106">
         <v>0</v>
@@ -32226,10 +32226,10 @@
         <v>31</v>
       </c>
       <c r="F107">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="G107">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="108" spans="1:7">
@@ -32249,7 +32249,7 @@
         <v>31</v>
       </c>
       <c r="F108">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="G108">
         <v>0</v>
@@ -32272,7 +32272,7 @@
         <v>31</v>
       </c>
       <c r="F109">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="G109">
         <v>0</v>
@@ -32295,7 +32295,7 @@
         <v>31</v>
       </c>
       <c r="F110">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="G110">
         <v>0</v>
@@ -32318,7 +32318,7 @@
         <v>31</v>
       </c>
       <c r="F111">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="G111">
         <v>0</v>
@@ -32341,10 +32341,10 @@
         <v>31</v>
       </c>
       <c r="F112">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="G112">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="113" spans="1:7">
@@ -32364,7 +32364,7 @@
         <v>31</v>
       </c>
       <c r="F113">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="G113">
         <v>0</v>
@@ -32387,10 +32387,10 @@
         <v>31</v>
       </c>
       <c r="F114">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G114">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="115" spans="1:7">
@@ -32410,10 +32410,10 @@
         <v>31</v>
       </c>
       <c r="F115">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="G115">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="116" spans="1:7">
@@ -32433,10 +32433,10 @@
         <v>31</v>
       </c>
       <c r="F116">
-        <v>73</v>
+        <v>51</v>
       </c>
       <c r="G116">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="117" spans="1:7">
@@ -32456,10 +32456,10 @@
         <v>31</v>
       </c>
       <c r="F117">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="G117">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="118" spans="1:7">
@@ -32479,10 +32479,10 @@
         <v>31</v>
       </c>
       <c r="F118">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="G118">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="119" spans="1:7">
@@ -32502,10 +32502,10 @@
         <v>31</v>
       </c>
       <c r="F119">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="G119">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="120" spans="1:7">
@@ -32525,10 +32525,10 @@
         <v>31</v>
       </c>
       <c r="F120">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="G120">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="121" spans="1:7">
@@ -32548,10 +32548,10 @@
         <v>31</v>
       </c>
       <c r="F121">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="G121">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="122" spans="1:7">
@@ -32571,10 +32571,10 @@
         <v>31</v>
       </c>
       <c r="F122">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="G122">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="123" spans="1:7">
@@ -32594,10 +32594,10 @@
         <v>31</v>
       </c>
       <c r="F123">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="G123">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="124" spans="1:7">
@@ -32617,10 +32617,10 @@
         <v>31</v>
       </c>
       <c r="F124">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="G124">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="125" spans="1:7">
@@ -32640,10 +32640,10 @@
         <v>31</v>
       </c>
       <c r="F125">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="G125">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="126" spans="1:7">
@@ -32663,10 +32663,10 @@
         <v>31</v>
       </c>
       <c r="F126">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="G126">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="127" spans="1:7">
@@ -32686,10 +32686,10 @@
         <v>31</v>
       </c>
       <c r="F127">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="G127">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="128" spans="1:7">
@@ -32709,10 +32709,10 @@
         <v>31</v>
       </c>
       <c r="F128">
-        <v>71</v>
+        <v>50</v>
       </c>
       <c r="G128">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="129" spans="1:7">
@@ -32732,10 +32732,10 @@
         <v>31</v>
       </c>
       <c r="F129">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="G129">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="130" spans="1:7">
@@ -32755,10 +32755,10 @@
         <v>31</v>
       </c>
       <c r="F130">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="G130">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="131" spans="1:7">
@@ -32778,10 +32778,10 @@
         <v>31</v>
       </c>
       <c r="F131">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="G131">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="132" spans="1:7">
@@ -32801,10 +32801,10 @@
         <v>31</v>
       </c>
       <c r="F132">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="G132">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="133" spans="1:7">
@@ -32824,10 +32824,10 @@
         <v>31</v>
       </c>
       <c r="F133">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="G133">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="134" spans="1:7">
@@ -32847,7 +32847,7 @@
         <v>32</v>
       </c>
       <c r="F134">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="G134">
         <v>0</v>
@@ -32870,7 +32870,7 @@
         <v>32</v>
       </c>
       <c r="F135">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G135">
         <v>0</v>
@@ -32893,7 +32893,7 @@
         <v>32</v>
       </c>
       <c r="F136">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="G136">
         <v>0</v>
@@ -32939,7 +32939,7 @@
         <v>32</v>
       </c>
       <c r="F138">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="G138">
         <v>0</v>
@@ -32962,7 +32962,7 @@
         <v>32</v>
       </c>
       <c r="F139">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G139">
         <v>0</v>
@@ -32985,7 +32985,7 @@
         <v>32</v>
       </c>
       <c r="F140">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G140">
         <v>0</v>
@@ -33008,7 +33008,7 @@
         <v>32</v>
       </c>
       <c r="F141">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="G141">
         <v>0</v>
@@ -33031,7 +33031,7 @@
         <v>32</v>
       </c>
       <c r="F142">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="G142">
         <v>0</v>
@@ -33054,7 +33054,7 @@
         <v>32</v>
       </c>
       <c r="F143">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="G143">
         <v>0</v>
@@ -33077,7 +33077,7 @@
         <v>32</v>
       </c>
       <c r="F144">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="G144">
         <v>0</v>
@@ -33100,7 +33100,7 @@
         <v>32</v>
       </c>
       <c r="F145">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="G145">
         <v>0</v>
@@ -33123,7 +33123,7 @@
         <v>32</v>
       </c>
       <c r="F146">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="G146">
         <v>0</v>
@@ -33146,7 +33146,7 @@
         <v>32</v>
       </c>
       <c r="F147">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="G147">
         <v>0</v>
@@ -33169,7 +33169,7 @@
         <v>32</v>
       </c>
       <c r="F148">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="G148">
         <v>0</v>
@@ -33192,10 +33192,10 @@
         <v>32</v>
       </c>
       <c r="F149">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G149">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="150" spans="1:7">
@@ -33215,7 +33215,7 @@
         <v>32</v>
       </c>
       <c r="F150">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="G150">
         <v>0</v>
@@ -33238,7 +33238,7 @@
         <v>32</v>
       </c>
       <c r="F151">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="G151">
         <v>0</v>
@@ -33261,7 +33261,7 @@
         <v>32</v>
       </c>
       <c r="F152">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="G152">
         <v>0</v>
@@ -33284,10 +33284,10 @@
         <v>32</v>
       </c>
       <c r="F153">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="G153">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="154" spans="1:7">
@@ -33307,7 +33307,7 @@
         <v>32</v>
       </c>
       <c r="F154">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="G154">
         <v>0</v>
@@ -33330,7 +33330,7 @@
         <v>32</v>
       </c>
       <c r="F155">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="G155">
         <v>0</v>
@@ -33353,7 +33353,7 @@
         <v>32</v>
       </c>
       <c r="F156">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G156">
         <v>0</v>
@@ -33376,7 +33376,7 @@
         <v>32</v>
       </c>
       <c r="F157">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="G157">
         <v>0</v>
@@ -33399,10 +33399,10 @@
         <v>32</v>
       </c>
       <c r="F158">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="G158">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="159" spans="1:7">
@@ -33422,7 +33422,7 @@
         <v>32</v>
       </c>
       <c r="F159">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="G159">
         <v>0</v>
@@ -33445,10 +33445,10 @@
         <v>32</v>
       </c>
       <c r="F160">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="G160">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="161" spans="1:7">
@@ -33468,7 +33468,7 @@
         <v>32</v>
       </c>
       <c r="F161">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="G161">
         <v>0</v>
@@ -33491,10 +33491,10 @@
         <v>32</v>
       </c>
       <c r="F162">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G162">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="163" spans="1:7">
@@ -33514,7 +33514,7 @@
         <v>32</v>
       </c>
       <c r="F163">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="G163">
         <v>0</v>
@@ -33537,7 +33537,7 @@
         <v>32</v>
       </c>
       <c r="F164">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="G164">
         <v>0</v>
@@ -33560,10 +33560,10 @@
         <v>32</v>
       </c>
       <c r="F165">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="G165">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="166" spans="1:7">
@@ -33583,10 +33583,10 @@
         <v>32</v>
       </c>
       <c r="F166">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="G166">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="167" spans="1:7">
@@ -33606,10 +33606,10 @@
         <v>33</v>
       </c>
       <c r="F167">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="G167">
-        <v>25</v>
+        <v>3</v>
       </c>
     </row>
     <row r="168" spans="1:7">
@@ -33629,10 +33629,10 @@
         <v>33</v>
       </c>
       <c r="F168">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="G168">
-        <v>25</v>
+        <v>3</v>
       </c>
     </row>
     <row r="169" spans="1:7">
@@ -33652,10 +33652,10 @@
         <v>33</v>
       </c>
       <c r="F169">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="G169">
-        <v>28</v>
+        <v>3</v>
       </c>
     </row>
     <row r="170" spans="1:7">
@@ -33675,10 +33675,10 @@
         <v>33</v>
       </c>
       <c r="F170">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="G170">
-        <v>28</v>
+        <v>3</v>
       </c>
     </row>
     <row r="171" spans="1:7">
@@ -33698,10 +33698,10 @@
         <v>33</v>
       </c>
       <c r="F171">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="G171">
-        <v>29</v>
+        <v>3</v>
       </c>
     </row>
     <row r="172" spans="1:7">
@@ -33721,10 +33721,10 @@
         <v>33</v>
       </c>
       <c r="F172">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="G172">
-        <v>21</v>
+        <v>3</v>
       </c>
     </row>
     <row r="173" spans="1:7">
@@ -33744,10 +33744,10 @@
         <v>33</v>
       </c>
       <c r="F173">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="G173">
-        <v>23</v>
+        <v>3</v>
       </c>
     </row>
     <row r="174" spans="1:7">
@@ -33767,10 +33767,10 @@
         <v>33</v>
       </c>
       <c r="F174">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="G174">
-        <v>28</v>
+        <v>3</v>
       </c>
     </row>
     <row r="175" spans="1:7">
@@ -33790,10 +33790,10 @@
         <v>33</v>
       </c>
       <c r="F175">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="G175">
-        <v>26</v>
+        <v>3</v>
       </c>
     </row>
     <row r="176" spans="1:7">
@@ -33813,10 +33813,10 @@
         <v>33</v>
       </c>
       <c r="F176">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="G176">
-        <v>21</v>
+        <v>3</v>
       </c>
     </row>
     <row r="177" spans="1:7">
@@ -33836,10 +33836,10 @@
         <v>33</v>
       </c>
       <c r="F177">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="G177">
-        <v>29</v>
+        <v>3</v>
       </c>
     </row>
     <row r="178" spans="1:7">
@@ -33859,10 +33859,10 @@
         <v>33</v>
       </c>
       <c r="F178">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="G178">
-        <v>32</v>
+        <v>3</v>
       </c>
     </row>
     <row r="179" spans="1:7">
@@ -33882,10 +33882,10 @@
         <v>33</v>
       </c>
       <c r="F179">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="G179">
-        <v>28</v>
+        <v>3</v>
       </c>
     </row>
     <row r="180" spans="1:7">
@@ -33905,10 +33905,10 @@
         <v>33</v>
       </c>
       <c r="F180">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="G180">
-        <v>34</v>
+        <v>3</v>
       </c>
     </row>
     <row r="181" spans="1:7">
@@ -33928,10 +33928,10 @@
         <v>33</v>
       </c>
       <c r="F181">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="G181">
-        <v>35</v>
+        <v>3</v>
       </c>
     </row>
     <row r="182" spans="1:7">
@@ -33951,10 +33951,10 @@
         <v>33</v>
       </c>
       <c r="F182">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="G182">
-        <v>27</v>
+        <v>3</v>
       </c>
     </row>
     <row r="183" spans="1:7">
@@ -33974,10 +33974,10 @@
         <v>33</v>
       </c>
       <c r="F183">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G183">
-        <v>26</v>
+        <v>3</v>
       </c>
     </row>
     <row r="184" spans="1:7">
@@ -33997,10 +33997,10 @@
         <v>33</v>
       </c>
       <c r="F184">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="G184">
-        <v>25</v>
+        <v>3</v>
       </c>
     </row>
     <row r="185" spans="1:7">
@@ -34020,10 +34020,10 @@
         <v>33</v>
       </c>
       <c r="F185">
-        <v>73</v>
+        <v>24</v>
       </c>
       <c r="G185">
-        <v>44</v>
+        <v>4</v>
       </c>
     </row>
     <row r="186" spans="1:7">
@@ -34043,10 +34043,10 @@
         <v>33</v>
       </c>
       <c r="F186">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="G186">
-        <v>25</v>
+        <v>3</v>
       </c>
     </row>
     <row r="187" spans="1:7">
@@ -34066,10 +34066,10 @@
         <v>33</v>
       </c>
       <c r="F187">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="G187">
-        <v>21</v>
+        <v>3</v>
       </c>
     </row>
     <row r="188" spans="1:7">
@@ -34089,10 +34089,10 @@
         <v>33</v>
       </c>
       <c r="F188">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="G188">
-        <v>21</v>
+        <v>3</v>
       </c>
     </row>
     <row r="189" spans="1:7">
@@ -34112,10 +34112,10 @@
         <v>33</v>
       </c>
       <c r="F189">
-        <v>52</v>
+        <v>29</v>
       </c>
       <c r="G189">
-        <v>33</v>
+        <v>3</v>
       </c>
     </row>
     <row r="190" spans="1:7">
@@ -34135,10 +34135,10 @@
         <v>33</v>
       </c>
       <c r="F190">
-        <v>52</v>
+        <v>31</v>
       </c>
       <c r="G190">
-        <v>39</v>
+        <v>4</v>
       </c>
     </row>
     <row r="191" spans="1:7">
@@ -34158,10 +34158,10 @@
         <v>33</v>
       </c>
       <c r="F191">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="G191">
-        <v>45</v>
+        <v>6</v>
       </c>
     </row>
     <row r="192" spans="1:7">
@@ -34181,10 +34181,10 @@
         <v>33</v>
       </c>
       <c r="F192">
-        <v>90</v>
+        <v>34</v>
       </c>
       <c r="G192">
-        <v>53</v>
+        <v>6</v>
       </c>
     </row>
     <row r="193" spans="1:7">
@@ -34204,10 +34204,10 @@
         <v>33</v>
       </c>
       <c r="F193">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="G193">
-        <v>48</v>
+        <v>5</v>
       </c>
     </row>
     <row r="194" spans="1:7">
@@ -34227,10 +34227,10 @@
         <v>33</v>
       </c>
       <c r="F194">
-        <v>64</v>
+        <v>31</v>
       </c>
       <c r="G194">
-        <v>36</v>
+        <v>3</v>
       </c>
     </row>
     <row r="195" spans="1:7">
@@ -34250,10 +34250,10 @@
         <v>33</v>
       </c>
       <c r="F195">
-        <v>68</v>
+        <v>32</v>
       </c>
       <c r="G195">
-        <v>41</v>
+        <v>4</v>
       </c>
     </row>
     <row r="196" spans="1:7">
@@ -34273,10 +34273,10 @@
         <v>33</v>
       </c>
       <c r="F196">
-        <v>92</v>
+        <v>26</v>
       </c>
       <c r="G196">
-        <v>41</v>
+        <v>4</v>
       </c>
     </row>
     <row r="197" spans="1:7">
@@ -34296,10 +34296,10 @@
         <v>33</v>
       </c>
       <c r="F197">
-        <v>56</v>
+        <v>22</v>
       </c>
       <c r="G197">
-        <v>31</v>
+        <v>3</v>
       </c>
     </row>
     <row r="198" spans="1:7">
@@ -34319,10 +34319,10 @@
         <v>33</v>
       </c>
       <c r="F198">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="G198">
-        <v>29</v>
+        <v>3</v>
       </c>
     </row>
     <row r="199" spans="1:7">
@@ -34342,10 +34342,10 @@
         <v>33</v>
       </c>
       <c r="F199">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="G199">
-        <v>23</v>
+        <v>3</v>
       </c>
     </row>
     <row r="200" spans="1:7">
@@ -34365,10 +34365,10 @@
         <v>34</v>
       </c>
       <c r="F200">
-        <v>32</v>
+        <v>54</v>
       </c>
       <c r="G200">
-        <v>34</v>
+        <v>7</v>
       </c>
     </row>
     <row r="201" spans="1:7">
@@ -34388,10 +34388,10 @@
         <v>34</v>
       </c>
       <c r="F201">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="G201">
-        <v>60</v>
+        <v>13</v>
       </c>
     </row>
     <row r="202" spans="1:7">
@@ -34411,10 +34411,10 @@
         <v>34</v>
       </c>
       <c r="F202">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="G202">
-        <v>28</v>
+        <v>6</v>
       </c>
     </row>
     <row r="203" spans="1:7">
@@ -34434,10 +34434,10 @@
         <v>34</v>
       </c>
       <c r="F203">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="G203">
-        <v>42</v>
+        <v>9</v>
       </c>
     </row>
     <row r="204" spans="1:7">
@@ -34457,10 +34457,10 @@
         <v>34</v>
       </c>
       <c r="F204">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="G204">
-        <v>22</v>
+        <v>5</v>
       </c>
     </row>
     <row r="205" spans="1:7">
@@ -34480,10 +34480,10 @@
         <v>34</v>
       </c>
       <c r="F205">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="G205">
-        <v>35</v>
+        <v>7</v>
       </c>
     </row>
     <row r="206" spans="1:7">
@@ -34503,10 +34503,10 @@
         <v>34</v>
       </c>
       <c r="F206">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="G206">
-        <v>64</v>
+        <v>13</v>
       </c>
     </row>
     <row r="207" spans="1:7">
@@ -34526,10 +34526,10 @@
         <v>34</v>
       </c>
       <c r="F207">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="G207">
-        <v>76</v>
+        <v>16</v>
       </c>
     </row>
     <row r="208" spans="1:7">
@@ -34549,10 +34549,10 @@
         <v>34</v>
       </c>
       <c r="F208">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="G208">
-        <v>59</v>
+        <v>12</v>
       </c>
     </row>
     <row r="209" spans="1:7">
@@ -34572,7 +34572,7 @@
         <v>34</v>
       </c>
       <c r="F209">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="G209">
         <v>0</v>
@@ -34595,10 +34595,10 @@
         <v>34</v>
       </c>
       <c r="F210">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="G210">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="211" spans="1:7">
@@ -34618,10 +34618,10 @@
         <v>34</v>
       </c>
       <c r="F211">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="G211">
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="212" spans="1:7">
@@ -34641,10 +34641,10 @@
         <v>34</v>
       </c>
       <c r="F212">
-        <v>12</v>
+        <v>52</v>
       </c>
       <c r="G212">
-        <v>37</v>
+        <v>8</v>
       </c>
     </row>
     <row r="213" spans="1:7">
@@ -34664,10 +34664,10 @@
         <v>34</v>
       </c>
       <c r="F213">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="G213">
-        <v>55</v>
+        <v>12</v>
       </c>
     </row>
     <row r="214" spans="1:7">
@@ -34687,10 +34687,10 @@
         <v>34</v>
       </c>
       <c r="F214">
-        <v>0</v>
+        <v>74</v>
       </c>
       <c r="G214">
-        <v>33</v>
+        <v>7</v>
       </c>
     </row>
     <row r="215" spans="1:7">
@@ -34710,10 +34710,10 @@
         <v>34</v>
       </c>
       <c r="F215">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="G215">
-        <v>30</v>
+        <v>6</v>
       </c>
     </row>
     <row r="216" spans="1:7">
@@ -34733,10 +34733,10 @@
         <v>34</v>
       </c>
       <c r="F216">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="G216">
-        <v>32</v>
+        <v>7</v>
       </c>
     </row>
     <row r="217" spans="1:7">
@@ -34756,10 +34756,10 @@
         <v>34</v>
       </c>
       <c r="F217">
-        <v>10</v>
+        <v>51</v>
       </c>
       <c r="G217">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="218" spans="1:7">
@@ -34779,10 +34779,10 @@
         <v>34</v>
       </c>
       <c r="F218">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="G218">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="219" spans="1:7">
@@ -34802,10 +34802,10 @@
         <v>34</v>
       </c>
       <c r="F219">
-        <v>10</v>
+        <v>59</v>
       </c>
       <c r="G219">
-        <v>15</v>
+        <v>3</v>
       </c>
     </row>
     <row r="220" spans="1:7">
@@ -34825,10 +34825,10 @@
         <v>34</v>
       </c>
       <c r="F220">
-        <v>12</v>
+        <v>52</v>
       </c>
       <c r="G220">
-        <v>17</v>
+        <v>4</v>
       </c>
     </row>
     <row r="221" spans="1:7">
@@ -34848,10 +34848,10 @@
         <v>34</v>
       </c>
       <c r="F221">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="G221">
-        <v>42</v>
+        <v>9</v>
       </c>
     </row>
     <row r="222" spans="1:7">
@@ -34871,10 +34871,10 @@
         <v>34</v>
       </c>
       <c r="F222">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="G222">
-        <v>21</v>
+        <v>4</v>
       </c>
     </row>
     <row r="223" spans="1:7">
@@ -34894,10 +34894,10 @@
         <v>34</v>
       </c>
       <c r="F223">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="G223">
-        <v>55</v>
+        <v>11</v>
       </c>
     </row>
     <row r="224" spans="1:7">
@@ -34917,10 +34917,10 @@
         <v>34</v>
       </c>
       <c r="F224">
-        <v>14</v>
+        <v>54</v>
       </c>
       <c r="G224">
-        <v>51</v>
+        <v>11</v>
       </c>
     </row>
     <row r="225" spans="1:7">
@@ -34940,10 +34940,10 @@
         <v>34</v>
       </c>
       <c r="F225">
-        <v>14</v>
+        <v>62</v>
       </c>
       <c r="G225">
-        <v>100</v>
+        <v>21</v>
       </c>
     </row>
     <row r="226" spans="1:7">
@@ -34963,10 +34963,10 @@
         <v>34</v>
       </c>
       <c r="F226">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="G226">
-        <v>34</v>
+        <v>7</v>
       </c>
     </row>
     <row r="227" spans="1:7">
@@ -34986,10 +34986,10 @@
         <v>34</v>
       </c>
       <c r="F227">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="G227">
-        <v>30</v>
+        <v>6</v>
       </c>
     </row>
     <row r="228" spans="1:7">
@@ -35009,10 +35009,10 @@
         <v>34</v>
       </c>
       <c r="F228">
-        <v>16</v>
+        <v>52</v>
       </c>
       <c r="G228">
-        <v>41</v>
+        <v>9</v>
       </c>
     </row>
     <row r="229" spans="1:7">
@@ -35032,7 +35032,7 @@
         <v>34</v>
       </c>
       <c r="F229">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="G229">
         <v>0</v>
@@ -35055,10 +35055,10 @@
         <v>34</v>
       </c>
       <c r="F230">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="G230">
-        <v>16</v>
+        <v>3</v>
       </c>
     </row>
     <row r="231" spans="1:7">
@@ -35078,10 +35078,10 @@
         <v>34</v>
       </c>
       <c r="F231">
-        <v>7</v>
+        <v>42</v>
       </c>
       <c r="G231">
-        <v>30</v>
+        <v>6</v>
       </c>
     </row>
     <row r="232" spans="1:7">
@@ -35101,10 +35101,10 @@
         <v>34</v>
       </c>
       <c r="F232">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="G232">
-        <v>43</v>
+        <v>9</v>
       </c>
     </row>
     <row r="233" spans="1:7">
@@ -35124,10 +35124,10 @@
         <v>35</v>
       </c>
       <c r="F233">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="G233">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="234" spans="1:7">
@@ -35147,10 +35147,10 @@
         <v>35</v>
       </c>
       <c r="F234">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="G234">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="235" spans="1:7">
@@ -35170,10 +35170,10 @@
         <v>35</v>
       </c>
       <c r="F235">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="G235">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="236" spans="1:7">
@@ -35193,7 +35193,7 @@
         <v>35</v>
       </c>
       <c r="F236">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="G236">
         <v>10</v>
@@ -35216,7 +35216,7 @@
         <v>35</v>
       </c>
       <c r="F237">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="G237">
         <v>9</v>
@@ -35239,7 +35239,7 @@
         <v>35</v>
       </c>
       <c r="F238">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G238">
         <v>9</v>
@@ -35262,10 +35262,10 @@
         <v>35</v>
       </c>
       <c r="F239">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="G239">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="240" spans="1:7">
@@ -35285,10 +35285,10 @@
         <v>35</v>
       </c>
       <c r="F240">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="G240">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="241" spans="1:7">
@@ -35308,7 +35308,7 @@
         <v>35</v>
       </c>
       <c r="F241">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="G241">
         <v>11</v>
@@ -35331,10 +35331,10 @@
         <v>35</v>
       </c>
       <c r="F242">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="G242">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="243" spans="1:7">
@@ -35354,10 +35354,10 @@
         <v>35</v>
       </c>
       <c r="F243">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="G243">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="244" spans="1:7">
@@ -35377,10 +35377,10 @@
         <v>35</v>
       </c>
       <c r="F244">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="G244">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="245" spans="1:7">
@@ -35400,10 +35400,10 @@
         <v>35</v>
       </c>
       <c r="F245">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="G245">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="246" spans="1:7">
@@ -35423,10 +35423,10 @@
         <v>35</v>
       </c>
       <c r="F246">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="G246">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="247" spans="1:7">
@@ -35446,10 +35446,10 @@
         <v>35</v>
       </c>
       <c r="F247">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="G247">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="248" spans="1:7">
@@ -35469,10 +35469,10 @@
         <v>35</v>
       </c>
       <c r="F248">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="G248">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="249" spans="1:7">
@@ -35492,7 +35492,7 @@
         <v>35</v>
       </c>
       <c r="F249">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="G249">
         <v>10</v>
@@ -35515,10 +35515,10 @@
         <v>35</v>
       </c>
       <c r="F250">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="G250">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="251" spans="1:7">
@@ -35538,7 +35538,7 @@
         <v>35</v>
       </c>
       <c r="F251">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="G251">
         <v>12</v>
@@ -35561,7 +35561,7 @@
         <v>35</v>
       </c>
       <c r="F252">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="G252">
         <v>13</v>
@@ -35584,10 +35584,10 @@
         <v>35</v>
       </c>
       <c r="F253">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="G253">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="254" spans="1:7">
@@ -35607,7 +35607,7 @@
         <v>35</v>
       </c>
       <c r="F254">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="G254">
         <v>11</v>
@@ -35630,10 +35630,10 @@
         <v>35</v>
       </c>
       <c r="F255">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="G255">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="256" spans="1:7">
@@ -35653,7 +35653,7 @@
         <v>35</v>
       </c>
       <c r="F256">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="G256">
         <v>14</v>
@@ -35676,10 +35676,10 @@
         <v>35</v>
       </c>
       <c r="F257">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="G257">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="258" spans="1:7">
@@ -35699,10 +35699,10 @@
         <v>35</v>
       </c>
       <c r="F258">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G258">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="259" spans="1:7">
@@ -35722,10 +35722,10 @@
         <v>35</v>
       </c>
       <c r="F259">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="G259">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="260" spans="1:7">
@@ -35745,10 +35745,10 @@
         <v>35</v>
       </c>
       <c r="F260">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="G260">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="261" spans="1:7">
@@ -35768,10 +35768,10 @@
         <v>35</v>
       </c>
       <c r="F261">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G261">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="262" spans="1:7">
@@ -35791,10 +35791,10 @@
         <v>35</v>
       </c>
       <c r="F262">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="G262">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="263" spans="1:7">
@@ -35814,7 +35814,7 @@
         <v>35</v>
       </c>
       <c r="F263">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="G263">
         <v>12</v>
@@ -35837,7 +35837,7 @@
         <v>35</v>
       </c>
       <c r="F264">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="G264">
         <v>11</v>
@@ -35860,7 +35860,7 @@
         <v>35</v>
       </c>
       <c r="F265">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="G265">
         <v>9</v>

</xml_diff>